<commit_message>
:lipstick: style(modelos): Pondo a logo da Diretoria de Projetos no cabeçalho dos modelos
</commit_message>
<xml_diff>
--- a/modelos/xlsx/01_canvas_de_ideacao.xlsx
+++ b/modelos/xlsx/01_canvas_de_ideacao.xlsx
@@ -288,7 +288,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1552575" cy="247650"/>
+    <ext cx="2047875" cy="247650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -318,7 +318,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1552575" cy="247650"/>
+    <ext cx="2047875" cy="247650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>

</xml_diff>